<commit_message>
Actualizacion automatica de datos - lun 13/07/2026 14:05:10,59
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Julio.xlsx
+++ b/Cronograma de Tareas/Cronograma Julio.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="92" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B49C3AEB-B14B-4C26-9E8E-68ECE1AC4F80}"/>
+  <xr:revisionPtr revIDLastSave="97" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB38A53F-F906-4E04-B2E4-15990395DB62}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 6 al 12 Jul" sheetId="10" r:id="rId1"/>
-    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId2"/>
+    <sheet name="Semana 2 - 13 al 19 Jul" sheetId="11" r:id="rId2"/>
+    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="84">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -311,6 +312,12 @@
   </si>
   <si>
     <t xml:space="preserve">Yefferson </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alexander </t>
+  </si>
+  <si>
+    <t>Revisión Usuarios Nivel 2 - CRM con TAG de Abuso de Bonos (15 días)</t>
   </si>
 </sst>
 </file>
@@ -465,7 +472,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -519,6 +526,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -526,7 +534,337 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="65">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1178,43 +1516,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41C7291A-7212-4757-A43C-50195386FDB5}">
   <dimension ref="B2:L41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.28515625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" style="2"/>
-    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15" style="2"/>
-    <col min="8" max="8" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15" style="2"/>
-    <col min="11" max="11" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="15" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="19" t="s">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B2" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="19"/>
+      <c r="C2" s="20"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="F2" s="19"/>
-      <c r="H2" s="19" t="s">
+      <c r="F2" s="20"/>
+      <c r="H2" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="I2" s="19"/>
-      <c r="K2" s="19" t="s">
+      <c r="I2" s="20"/>
+      <c r="K2" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="L2" s="19"/>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L2" s="20"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3" s="13" t="s">
         <v>0</v>
       </c>
@@ -1241,7 +1579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
@@ -1267,7 +1605,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
@@ -1293,7 +1631,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>66</v>
       </c>
@@ -1319,7 +1657,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
@@ -1345,7 +1683,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
@@ -1371,7 +1709,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
@@ -1397,7 +1735,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H10" s="5" t="s">
         <v>15</v>
       </c>
@@ -1411,15 +1749,15 @@
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="19" t="s">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B11" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="E11" s="19" t="s">
+      <c r="C11" s="20"/>
+      <c r="E11" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="F11" s="19"/>
+      <c r="F11" s="20"/>
       <c r="H11" s="5" t="s">
         <v>7</v>
       </c>
@@ -1433,7 +1771,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="13" t="s">
         <v>0</v>
       </c>
@@ -1459,7 +1797,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>10</v>
       </c>
@@ -1486,7 +1824,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>12</v>
       </c>
@@ -1513,7 +1851,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>15</v>
       </c>
@@ -1539,7 +1877,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>21</v>
       </c>
@@ -1555,7 +1893,7 @@
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B17" s="12" t="s">
         <v>22</v>
       </c>
@@ -1568,16 +1906,16 @@
       <c r="F17" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="H17" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="I17" s="19"/>
-      <c r="K17" s="19" t="s">
+      <c r="I17" s="20"/>
+      <c r="K17" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="L17" s="19"/>
-    </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L17" s="20"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="8" t="s">
         <v>60</v>
       </c>
@@ -1603,7 +1941,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H19" s="5" t="s">
         <v>10</v>
       </c>
@@ -1617,15 +1955,15 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="19" t="s">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B20" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="C20" s="19"/>
-      <c r="E20" s="19" t="s">
+      <c r="C20" s="20"/>
+      <c r="E20" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F20" s="19"/>
+      <c r="F20" s="20"/>
       <c r="H20" s="5" t="s">
         <v>12</v>
       </c>
@@ -1639,7 +1977,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="13" t="s">
         <v>0</v>
       </c>
@@ -1665,7 +2003,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="8" t="s">
         <v>28</v>
       </c>
@@ -1691,7 +2029,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="8" t="s">
         <v>30</v>
       </c>
@@ -1717,7 +2055,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="8" t="s">
         <v>26</v>
       </c>
@@ -1743,7 +2081,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="8" t="s">
         <v>31</v>
       </c>
@@ -1769,7 +2107,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
         <v>20</v>
       </c>
@@ -1795,7 +2133,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
         <v>34</v>
       </c>
@@ -1815,7 +2153,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="5" t="s">
         <v>19</v>
       </c>
@@ -1835,7 +2173,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="5" t="s">
         <v>64</v>
       </c>
@@ -1843,23 +2181,23 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
         <v>32</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="H30" s="19" t="s">
+      <c r="H30" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="I30" s="19"/>
-      <c r="K30" s="19" t="s">
+      <c r="I30" s="20"/>
+      <c r="K30" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="L30" s="19"/>
-    </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L30" s="20"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31"/>
       <c r="C31"/>
       <c r="H31" s="13" t="s">
@@ -1875,7 +2213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32"/>
       <c r="C32"/>
       <c r="D32"/>
@@ -1892,7 +2230,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33"/>
       <c r="C33"/>
       <c r="D33"/>
@@ -1909,7 +2247,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34"/>
       <c r="C34"/>
       <c r="D34"/>
@@ -1926,7 +2264,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35"/>
       <c r="C35"/>
       <c r="D35"/>
@@ -1943,7 +2281,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36"/>
       <c r="C36"/>
       <c r="D36"/>
@@ -1960,154 +2298,1084 @@
         <v>24</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37"/>
       <c r="C37"/>
       <c r="D37"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38"/>
       <c r="C38"/>
       <c r="D38"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39"/>
       <c r="C39"/>
       <c r="D39"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40"/>
       <c r="C40"/>
       <c r="D40"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D41"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="31" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="30" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="29" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B25">
-    <cfRule type="duplicateValues" dxfId="28" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28 B26">
-    <cfRule type="duplicateValues" dxfId="27" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29 B27 B9">
-    <cfRule type="duplicateValues" dxfId="26" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="25" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="24" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="23" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="22" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="21" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="20" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="19" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="18" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="17" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="16" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="15" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="14" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="13" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="12" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="10" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="9" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="8" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="7" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="6" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="5" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="3" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="2" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="1" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E66C14E4-1304-4127-AC7E-50C32F1AE060}">
+  <dimension ref="B2:L41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="56.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7" style="2" customWidth="1"/>
+    <col min="5" max="5" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.88671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="15" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B2" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="F2" s="20"/>
+      <c r="H2" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="I2" s="20"/>
+      <c r="K2" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="L2" s="20"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="L4" s="14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B6" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="E10" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B11" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="H11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B12" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" s="20"/>
+      <c r="H12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L13" s="14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L14" s="14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B15" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="L16" s="1"/>
+    </row>
+    <row r="17" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B17" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H17" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="I17" s="20"/>
+      <c r="K17" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="L17" s="20"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B18" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="L18" s="15" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B20" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="E21" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F21" s="20"/>
+      <c r="H21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B22" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="20"/>
+      <c r="E22" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B23" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B24" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B25" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B26" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B27" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="K27" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B28" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K28" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B29" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B30" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H30" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="I30" s="20"/>
+      <c r="K30" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="L30" s="20"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B31"/>
+      <c r="C31"/>
+      <c r="H31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="L31" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B32"/>
+      <c r="C32"/>
+      <c r="D32"/>
+      <c r="H32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L32" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B33"/>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="H33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L33" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B34"/>
+      <c r="C34"/>
+      <c r="D34"/>
+      <c r="H34" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L34" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B35"/>
+      <c r="C35"/>
+      <c r="D35"/>
+      <c r="H35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L35" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B36"/>
+      <c r="C36"/>
+      <c r="D36"/>
+      <c r="H36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L36" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B38"/>
+      <c r="C38"/>
+      <c r="D38"/>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B39"/>
+      <c r="C39"/>
+      <c r="D39"/>
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="D40"/>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="D41"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="duplicateValues" dxfId="32" priority="30"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7">
+    <cfRule type="duplicateValues" dxfId="31" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="duplicateValues" dxfId="30" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19">
+    <cfRule type="duplicateValues" dxfId="29" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B24:B26 B20">
+    <cfRule type="duplicateValues" dxfId="28" priority="32"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B28 B9">
+    <cfRule type="duplicateValues" dxfId="27" priority="33"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29 B27">
+    <cfRule type="duplicateValues" dxfId="26" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6">
+    <cfRule type="duplicateValues" dxfId="25" priority="24"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="duplicateValues" dxfId="24" priority="23"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8">
+    <cfRule type="duplicateValues" dxfId="23" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="duplicateValues" dxfId="22" priority="27"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E18">
+    <cfRule type="duplicateValues" dxfId="21" priority="17"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E19">
+    <cfRule type="duplicateValues" dxfId="20" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E26">
+    <cfRule type="duplicateValues" dxfId="19" priority="15"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E27">
+    <cfRule type="duplicateValues" dxfId="18" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="duplicateValues" dxfId="17" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="duplicateValues" dxfId="16" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="duplicateValues" dxfId="15" priority="20"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="duplicateValues" dxfId="14" priority="28"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24">
+    <cfRule type="duplicateValues" dxfId="13" priority="12"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
+    <cfRule type="duplicateValues" dxfId="12" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="duplicateValues" dxfId="10" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="duplicateValues" dxfId="9" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4">
+    <cfRule type="duplicateValues" dxfId="8" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
+    <cfRule type="duplicateValues" dxfId="7" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12">
+    <cfRule type="duplicateValues" dxfId="6" priority="18"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K13">
+    <cfRule type="duplicateValues" dxfId="5" priority="29"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K23">
+    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K24">
+    <cfRule type="duplicateValues" dxfId="3" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K25">
+    <cfRule type="duplicateValues" dxfId="2" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K35">
+    <cfRule type="duplicateValues" dxfId="1" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K36">
+    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5EE4785-03B3-42C8-BF36-D812A392D9B8}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="95.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="95.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="47.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="94.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="94.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>35</v>
       </c>
@@ -2115,7 +3383,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>6</v>
       </c>
@@ -2123,7 +3391,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2131,7 +3399,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>9</v>
       </c>
@@ -2139,7 +3407,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>20</v>
       </c>
@@ -2147,7 +3415,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>19</v>
       </c>
@@ -2155,7 +3423,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>7</v>
       </c>
@@ -2163,7 +3431,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>43</v>
       </c>
@@ -2171,7 +3439,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>8</v>
       </c>
@@ -2179,7 +3447,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>14</v>
       </c>
@@ -2187,7 +3455,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>12</v>
       </c>
@@ -2195,7 +3463,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>61</v>
       </c>
@@ -2203,7 +3471,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>21</v>
       </c>
@@ -2211,7 +3479,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>48</v>
       </c>
@@ -2219,7 +3487,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>10</v>
       </c>
@@ -2227,7 +3495,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>26</v>
       </c>
@@ -2235,7 +3503,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
         <v>32</v>
       </c>
@@ -2243,7 +3511,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
         <v>30</v>
       </c>
@@ -2251,7 +3519,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
         <v>34</v>
       </c>
@@ -2259,7 +3527,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="150" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="144" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
         <v>28</v>
       </c>
@@ -2267,7 +3535,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>31</v>
       </c>
@@ -2275,7 +3543,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>27</v>
       </c>
@@ -2283,7 +3551,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
         <v>18</v>
       </c>
@@ -2291,7 +3559,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A24" s="10" t="s">
         <v>11</v>
       </c>
@@ -2299,7 +3567,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="10" t="s">
         <v>64</v>
       </c>
@@ -2314,21 +3582,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -2529,10 +3782,36 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2555,20 +3834,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - jue 16/07/2026 18:02:40,08
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Julio.xlsx
+++ b/Cronograma de Tareas/Cronograma Julio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="97" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB38A53F-F906-4E04-B2E4-15990395DB62}"/>
+  <xr:revisionPtr revIDLastSave="98" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FACD53B6-537E-40DE-8E54-19478C14D193}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView minimized="1" xWindow="-8460" yWindow="2940" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 6 al 12 Jul" sheetId="10" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="84">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -2323,18 +2323,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="64" priority="30"/>
@@ -2824,7 +2824,7 @@
         <v>13</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>29</v>
@@ -2846,7 +2846,7 @@
         <v>4</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>29</v>
@@ -2871,12 +2871,6 @@
       <c r="C19" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E19" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>29</v>
-      </c>
       <c r="H19" s="5" t="s">
         <v>10</v>
       </c>
@@ -2897,6 +2891,10 @@
       <c r="C20" s="4" t="s">
         <v>13</v>
       </c>
+      <c r="E20" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" s="20"/>
       <c r="H20" s="5" t="s">
         <v>12</v>
       </c>
@@ -2911,10 +2909,12 @@
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="E21" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="F21" s="20"/>
+      <c r="E21" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>1</v>
+      </c>
       <c r="H21" s="3" t="s">
         <v>3</v>
       </c>
@@ -2933,11 +2933,11 @@
         <v>69</v>
       </c>
       <c r="C22" s="20"/>
-      <c r="E22" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>1</v>
+      <c r="E22" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>6</v>
@@ -2960,7 +2960,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>24</v>
@@ -2986,7 +2986,7 @@
         <v>25</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>24</v>
@@ -3012,7 +3012,7 @@
         <v>25</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>24</v>
@@ -3038,7 +3038,7 @@
         <v>59</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>24</v>
@@ -3062,12 +3062,6 @@
       </c>
       <c r="C27" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>24</v>
       </c>
       <c r="H27" s="6" t="s">
         <v>19</v>
@@ -3258,7 +3252,7 @@
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="E20:F20"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
@@ -3296,16 +3290,16 @@
   <conditionalFormatting sqref="E9">
     <cfRule type="duplicateValues" dxfId="22" priority="27"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E17">
+    <cfRule type="duplicateValues" dxfId="21" priority="17"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="21" priority="17"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E19">
     <cfRule type="duplicateValues" dxfId="20" priority="16"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E25">
+    <cfRule type="duplicateValues" dxfId="19" priority="15"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="19" priority="15"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E27">
     <cfRule type="duplicateValues" dxfId="18" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
@@ -3783,18 +3777,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3817,6 +3811,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -3831,12 +3833,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - vie 17/07/2026 17:47:53,99
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Julio.xlsx
+++ b/Cronograma de Tareas/Cronograma Julio.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="98" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FACD53B6-537E-40DE-8E54-19478C14D193}"/>
+  <xr:revisionPtr revIDLastSave="101" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A9595E1-8818-4256-979A-B41AFB01E151}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="-8460" yWindow="2940" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 6 al 12 Jul" sheetId="10" r:id="rId1"/>
     <sheet name="Semana 2 - 13 al 19 Jul" sheetId="11" r:id="rId2"/>
-    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId3"/>
+    <sheet name="Semana 3 - 20 al 26 Jul" sheetId="12" r:id="rId3"/>
+    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="84">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -534,7 +535,337 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="65">
+  <dxfs count="98">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2323,114 +2654,114 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="64" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="63" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="62" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B25">
-    <cfRule type="duplicateValues" dxfId="61" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28 B26">
-    <cfRule type="duplicateValues" dxfId="60" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29 B27 B9">
-    <cfRule type="duplicateValues" dxfId="59" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="58" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="57" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="56" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="55" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="54" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="53" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="52" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="51" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="50" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="49" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="48" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="47" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="46" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="45" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="44" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="43" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="42" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="41" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="40" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="39" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="38" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="37" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="36" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="35" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="34" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="33" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3258,109 +3589,1033 @@
     <mergeCell ref="E2:F2"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="32" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="31" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="30" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19">
-    <cfRule type="duplicateValues" dxfId="29" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24:B26 B20">
-    <cfRule type="duplicateValues" dxfId="28" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28 B9">
-    <cfRule type="duplicateValues" dxfId="27" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29 B27">
-    <cfRule type="duplicateValues" dxfId="26" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="25" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="24" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="23" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="22" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="21" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="20" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="19" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="18" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="17" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="16" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="15" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="14" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="13" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="12" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="10" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="9" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="8" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="7" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="6" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="5" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="3" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="2" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="1" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{784A59EB-EBFC-4A2F-9CB8-F88987B32B22}">
+  <dimension ref="B2:L41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="56.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" style="2" customWidth="1"/>
+    <col min="5" max="5" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.88671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="15" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B2" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="F2" s="20"/>
+      <c r="H2" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="I2" s="20"/>
+      <c r="K2" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="L2" s="20"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="L4" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B6" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="H10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B11" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="E11" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="20"/>
+      <c r="H11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B12" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L13" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L14" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B15" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="L16" s="1"/>
+    </row>
+    <row r="17" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B17" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="I17" s="20"/>
+      <c r="K17" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="L17" s="20"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B18" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="L18" s="15" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B20" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" s="20"/>
+      <c r="E20" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" s="20"/>
+      <c r="H20" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B21" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B22" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B23" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B24" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B25" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B26" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B27" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K27" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B28" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K28" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B29" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B30" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H30" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="I30" s="20"/>
+      <c r="K30" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="L30" s="20"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B31" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="L31" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B32"/>
+      <c r="C32"/>
+      <c r="D32"/>
+      <c r="H32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L32" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B33"/>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="H33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L33" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B34"/>
+      <c r="C34"/>
+      <c r="D34"/>
+      <c r="H34" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L34" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B35"/>
+      <c r="C35"/>
+      <c r="D35"/>
+      <c r="H35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L35" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B36"/>
+      <c r="C36"/>
+      <c r="D36"/>
+      <c r="H36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L36" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="D38"/>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="D39"/>
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="D40"/>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="D41"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="duplicateValues" dxfId="32" priority="30"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7">
+    <cfRule type="duplicateValues" dxfId="31" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="duplicateValues" dxfId="30" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30">
+    <cfRule type="duplicateValues" dxfId="29" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29 B22:B24">
+    <cfRule type="duplicateValues" dxfId="28" priority="32"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B26 B9">
+    <cfRule type="duplicateValues" dxfId="27" priority="33"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B27 B25">
+    <cfRule type="duplicateValues" dxfId="26" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6">
+    <cfRule type="duplicateValues" dxfId="25" priority="24"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="duplicateValues" dxfId="24" priority="23"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8">
+    <cfRule type="duplicateValues" dxfId="23" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="duplicateValues" dxfId="22" priority="27"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17">
+    <cfRule type="duplicateValues" dxfId="21" priority="17"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E18">
+    <cfRule type="duplicateValues" dxfId="20" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25">
+    <cfRule type="duplicateValues" dxfId="19" priority="15"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E26">
+    <cfRule type="duplicateValues" dxfId="18" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="duplicateValues" dxfId="17" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="duplicateValues" dxfId="16" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="duplicateValues" dxfId="15" priority="20"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="duplicateValues" dxfId="14" priority="28"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24">
+    <cfRule type="duplicateValues" dxfId="13" priority="12"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
+    <cfRule type="duplicateValues" dxfId="12" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="duplicateValues" dxfId="10" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="duplicateValues" dxfId="9" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4">
+    <cfRule type="duplicateValues" dxfId="8" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
+    <cfRule type="duplicateValues" dxfId="7" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12">
+    <cfRule type="duplicateValues" dxfId="6" priority="18"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K13">
+    <cfRule type="duplicateValues" dxfId="5" priority="29"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K23">
+    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K24">
+    <cfRule type="duplicateValues" dxfId="3" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K25">
+    <cfRule type="duplicateValues" dxfId="2" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K35">
+    <cfRule type="duplicateValues" dxfId="1" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K36">
+    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5EE4785-03B3-42C8-BF36-D812A392D9B8}">
   <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="95.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3576,6 +4831,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -3776,22 +5046,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3808,29 +5088,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - sáb 18/07/2026 18:54:12,90
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Julio.xlsx
+++ b/Cronograma de Tareas/Cronograma Julio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A9595E1-8818-4256-979A-B41AFB01E151}"/>
+  <xr:revisionPtr revIDLastSave="103" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1ACA437-7636-4043-95DD-E979524E0228}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 6 al 12 Jul" sheetId="10" r:id="rId1"/>
@@ -2654,18 +2654,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="97" priority="30"/>
@@ -3475,7 +3475,7 @@
         <v>10</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="K32" s="5" t="s">
         <v>10</v>
@@ -3492,7 +3492,7 @@
         <v>12</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="K33" s="5" t="s">
         <v>12</v>
@@ -3509,7 +3509,7 @@
         <v>27</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="K34" s="5" t="s">
         <v>27</v>
@@ -3526,7 +3526,7 @@
         <v>19</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="K35" s="5" t="s">
         <v>19</v>
@@ -3543,7 +3543,7 @@
         <v>20</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="K36" s="5" t="s">
         <v>20</v>
@@ -4499,18 +4499,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="32" priority="30"/>
@@ -4521,17 +4521,17 @@
   <conditionalFormatting sqref="B8">
     <cfRule type="duplicateValues" dxfId="30" priority="25"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B26 B9">
+    <cfRule type="duplicateValues" dxfId="29" priority="33"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B27 B25">
+    <cfRule type="duplicateValues" dxfId="28" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29 B22:B24">
+    <cfRule type="duplicateValues" dxfId="27" priority="32"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="29" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B29 B22:B24">
-    <cfRule type="duplicateValues" dxfId="28" priority="32"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B26 B9">
-    <cfRule type="duplicateValues" dxfId="27" priority="33"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B27 B25">
-    <cfRule type="duplicateValues" dxfId="26" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
     <cfRule type="duplicateValues" dxfId="25" priority="24"/>
@@ -4831,21 +4831,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -5046,32 +5031,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5088,4 +5063,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - sáb 18/07/2026 21:21:11,01
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Julio.xlsx
+++ b/Cronograma de Tareas/Cronograma Julio.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1ACA437-7636-4043-95DD-E979524E0228}"/>
+  <xr:revisionPtr revIDLastSave="106" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{285DB50A-DF2E-48E1-8752-39A1C9B25204}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
@@ -1846,6 +1846,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41C7291A-7212-4757-A43C-50195386FDB5}">
+  <sheetPr codeName="Hoja1"/>
   <dimension ref="B2:L41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2769,6 +2770,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E66C14E4-1304-4127-AC7E-50C32F1AE060}">
+  <sheetPr codeName="Hoja2"/>
   <dimension ref="B2:L41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3212,7 +3214,7 @@
         <v>10</v>
       </c>
       <c r="L19" s="4" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.3">
@@ -3280,7 +3282,7 @@
         <v>3</v>
       </c>
       <c r="L22" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.3">
@@ -3306,7 +3308,7 @@
         <v>14</v>
       </c>
       <c r="L23" s="4" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.3">
@@ -3332,7 +3334,7 @@
         <v>7</v>
       </c>
       <c r="L24" s="4" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.3">
@@ -3404,7 +3406,7 @@
         <v>19</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.3">
@@ -3424,7 +3426,7 @@
         <v>20</v>
       </c>
       <c r="L28" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.3">
@@ -3693,6 +3695,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{784A59EB-EBFC-4A2F-9CB8-F88987B32B22}">
+  <sheetPr codeName="Hoja3"/>
   <dimension ref="B2:L41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4617,6 +4620,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5EE4785-03B3-42C8-BF36-D812A392D9B8}">
+  <sheetPr codeName="Hoja4"/>
   <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="95.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
Actualizacion automatica de datos - lun 27/07/2026 15:24:23,30
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Julio.xlsx
+++ b/Cronograma de Tareas/Cronograma Julio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="109" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19495F36-EBAA-4256-9DD0-D566B162587D}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AD3C06B-D3A5-469F-9D12-146835E6C5F7}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="3" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 6 al 12 Jul" sheetId="10" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="84">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -2179,24 +2179,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41C7291A-7212-4757-A43C-50195386FDB5}">
   <sheetPr codeName="Hoja1"/>
   <dimension ref="B2:L41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.28515625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" style="2"/>
-    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15" style="2"/>
-    <col min="8" max="8" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15" style="2"/>
-    <col min="11" max="11" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="15" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B2" s="20" t="s">
         <v>67</v>
       </c>
@@ -2215,7 +2215,7 @@
       </c>
       <c r="L2" s="20"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3" s="13" t="s">
         <v>0</v>
       </c>
@@ -2242,7 +2242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
@@ -2268,7 +2268,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>66</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
@@ -2372,7 +2372,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H10" s="5" t="s">
         <v>15</v>
       </c>
@@ -2412,7 +2412,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="20" t="s">
         <v>68</v>
       </c>
@@ -2434,7 +2434,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="13" t="s">
         <v>0</v>
       </c>
@@ -2460,7 +2460,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>10</v>
       </c>
@@ -2487,7 +2487,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>12</v>
       </c>
@@ -2514,7 +2514,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>15</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>21</v>
       </c>
@@ -2556,7 +2556,7 @@
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B17" s="12" t="s">
         <v>22</v>
       </c>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="L17" s="20"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="8" t="s">
         <v>60</v>
       </c>
@@ -2604,7 +2604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H19" s="5" t="s">
         <v>10</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="20" t="s">
         <v>69</v>
       </c>
@@ -2640,7 +2640,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="13" t="s">
         <v>0</v>
       </c>
@@ -2666,7 +2666,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="8" t="s">
         <v>28</v>
       </c>
@@ -2692,7 +2692,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="8" t="s">
         <v>30</v>
       </c>
@@ -2718,7 +2718,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="8" t="s">
         <v>26</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="8" t="s">
         <v>31</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
         <v>20</v>
       </c>
@@ -2796,7 +2796,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
         <v>34</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="5" t="s">
         <v>19</v>
       </c>
@@ -2836,7 +2836,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="5" t="s">
         <v>64</v>
       </c>
@@ -2844,7 +2844,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
         <v>32</v>
       </c>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="L30" s="20"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31"/>
       <c r="C31"/>
       <c r="H31" s="13" t="s">
@@ -2876,7 +2876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32"/>
       <c r="C32"/>
       <c r="D32"/>
@@ -2893,7 +2893,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33"/>
       <c r="C33"/>
       <c r="D33"/>
@@ -2910,7 +2910,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34"/>
       <c r="C34"/>
       <c r="D34"/>
@@ -2927,7 +2927,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35"/>
       <c r="C35"/>
       <c r="D35"/>
@@ -2944,7 +2944,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36"/>
       <c r="C36"/>
       <c r="D36"/>
@@ -2961,43 +2961,43 @@
         <v>24</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37"/>
       <c r="C37"/>
       <c r="D37"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38"/>
       <c r="C38"/>
       <c r="D38"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39"/>
       <c r="C39"/>
       <c r="D39"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40"/>
       <c r="C40"/>
       <c r="D40"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D41"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="130" priority="30"/>
@@ -3103,24 +3103,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E66C14E4-1304-4127-AC7E-50C32F1AE060}">
   <sheetPr codeName="Hoja2"/>
   <dimension ref="B2:L41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="56.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="56.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="1" customWidth="1"/>
     <col min="4" max="4" width="7" style="2" customWidth="1"/>
-    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.85546875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.42578125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.88671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="15" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B2" s="20" t="s">
         <v>67</v>
       </c>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="L2" s="20"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3" s="13" t="s">
         <v>0</v>
       </c>
@@ -3166,7 +3166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
@@ -3192,7 +3192,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
@@ -3218,7 +3218,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>66</v>
       </c>
@@ -3244,7 +3244,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
@@ -3270,7 +3270,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
@@ -3296,7 +3296,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="E10" s="5" t="s">
         <v>32</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="20" t="s">
         <v>68</v>
       </c>
@@ -3360,7 +3360,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="13" t="s">
         <v>0</v>
       </c>
@@ -3384,7 +3384,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>10</v>
       </c>
@@ -3411,7 +3411,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>12</v>
       </c>
@@ -3438,7 +3438,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>15</v>
       </c>
@@ -3464,7 +3464,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>21</v>
       </c>
@@ -3480,7 +3480,7 @@
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B17" s="12" t="s">
         <v>22</v>
       </c>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="L17" s="20"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="8" t="s">
         <v>60</v>
       </c>
@@ -3528,7 +3528,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="5" t="s">
         <v>64</v>
       </c>
@@ -3548,7 +3548,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="8" t="s">
         <v>31</v>
       </c>
@@ -3572,7 +3572,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="E21" s="13" t="s">
         <v>23</v>
       </c>
@@ -3592,7 +3592,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="20" t="s">
         <v>69</v>
       </c>
@@ -3616,7 +3616,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="13" t="s">
         <v>0</v>
       </c>
@@ -3642,7 +3642,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="8" t="s">
         <v>28</v>
       </c>
@@ -3668,7 +3668,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="8" t="s">
         <v>30</v>
       </c>
@@ -3694,7 +3694,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="8" t="s">
         <v>26</v>
       </c>
@@ -3720,7 +3720,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
         <v>20</v>
       </c>
@@ -3740,7 +3740,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="5" t="s">
         <v>34</v>
       </c>
@@ -3760,7 +3760,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="5" t="s">
         <v>19</v>
       </c>
@@ -3768,7 +3768,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="19" t="s">
         <v>83</v>
       </c>
@@ -3784,7 +3784,7 @@
       </c>
       <c r="L30" s="20"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31"/>
       <c r="C31"/>
       <c r="H31" s="13" t="s">
@@ -3800,7 +3800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32"/>
       <c r="C32"/>
       <c r="D32"/>
@@ -3817,7 +3817,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33"/>
       <c r="C33"/>
       <c r="D33"/>
@@ -3834,7 +3834,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34"/>
       <c r="C34"/>
       <c r="D34"/>
@@ -3851,7 +3851,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35"/>
       <c r="C35"/>
       <c r="D35"/>
@@ -3868,7 +3868,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36"/>
       <c r="C36"/>
       <c r="D36"/>
@@ -3885,25 +3885,25 @@
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37"/>
       <c r="C37"/>
       <c r="D37"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38"/>
       <c r="C38"/>
       <c r="D38"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39"/>
       <c r="C39"/>
       <c r="D39"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D40"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D41"/>
     </row>
   </sheetData>
@@ -4028,24 +4028,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{784A59EB-EBFC-4A2F-9CB8-F88987B32B22}">
   <sheetPr codeName="Hoja3"/>
   <dimension ref="B2:L41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="56.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="56.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7" style="2" customWidth="1"/>
-    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.85546875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.42578125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.88671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="9" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="15" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B2" s="20" t="s">
         <v>67</v>
       </c>
@@ -4064,7 +4064,7 @@
       </c>
       <c r="L2" s="20"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3" s="13" t="s">
         <v>0</v>
       </c>
@@ -4091,7 +4091,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
@@ -4117,7 +4117,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
@@ -4143,7 +4143,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>66</v>
       </c>
@@ -4169,7 +4169,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
@@ -4195,7 +4195,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
@@ -4221,7 +4221,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
@@ -4247,7 +4247,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H10" s="5" t="s">
         <v>15</v>
       </c>
@@ -4261,7 +4261,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="20" t="s">
         <v>68</v>
       </c>
@@ -4283,7 +4283,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="13" t="s">
         <v>0</v>
       </c>
@@ -4309,7 +4309,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>10</v>
       </c>
@@ -4336,7 +4336,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>12</v>
       </c>
@@ -4363,7 +4363,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>15</v>
       </c>
@@ -4389,7 +4389,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>21</v>
       </c>
@@ -4405,7 +4405,7 @@
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B17" s="12" t="s">
         <v>22</v>
       </c>
@@ -4427,7 +4427,7 @@
       </c>
       <c r="L17" s="20"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="8" t="s">
         <v>60</v>
       </c>
@@ -4453,7 +4453,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H19" s="5" t="s">
         <v>10</v>
       </c>
@@ -4467,7 +4467,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="20" t="s">
         <v>69</v>
       </c>
@@ -4489,7 +4489,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="13" t="s">
         <v>0</v>
       </c>
@@ -4515,7 +4515,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="8" t="s">
         <v>28</v>
       </c>
@@ -4541,7 +4541,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="8" t="s">
         <v>30</v>
       </c>
@@ -4567,7 +4567,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="8" t="s">
         <v>26</v>
       </c>
@@ -4593,7 +4593,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="5" t="s">
         <v>20</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
         <v>34</v>
       </c>
@@ -4645,7 +4645,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
         <v>19</v>
       </c>
@@ -4665,7 +4665,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="19" t="s">
         <v>83</v>
       </c>
@@ -4685,7 +4685,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="8" t="s">
         <v>31</v>
       </c>
@@ -4693,7 +4693,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
         <v>64</v>
       </c>
@@ -4709,7 +4709,7 @@
       </c>
       <c r="L30" s="20"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="5" t="s">
         <v>32</v>
       </c>
@@ -4729,7 +4729,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32"/>
       <c r="C32"/>
       <c r="D32"/>
@@ -4746,7 +4746,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33"/>
       <c r="C33"/>
       <c r="D33"/>
@@ -4763,7 +4763,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34"/>
       <c r="C34"/>
       <c r="D34"/>
@@ -4780,7 +4780,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35"/>
       <c r="C35"/>
       <c r="D35"/>
@@ -4797,7 +4797,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36"/>
       <c r="C36"/>
       <c r="D36"/>
@@ -4814,37 +4814,37 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37"/>
       <c r="C37"/>
       <c r="D37"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D38"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D39"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D40"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D41"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="65" priority="30"/>
@@ -4952,24 +4952,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBBE273B-746A-447C-B291-AD69B002CBF8}">
   <dimension ref="B2:L41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="56.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="56.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7" style="2" customWidth="1"/>
-    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.85546875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.42578125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.88671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.88671875" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="15" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B2" s="20" t="s">
         <v>67</v>
       </c>
@@ -4988,7 +4988,7 @@
       </c>
       <c r="L2" s="20"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3" s="13" t="s">
         <v>0</v>
       </c>
@@ -5015,7 +5015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
@@ -5041,7 +5041,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
@@ -5067,7 +5067,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>66</v>
       </c>
@@ -5093,7 +5093,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
@@ -5119,7 +5119,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
@@ -5145,7 +5145,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
@@ -5171,7 +5171,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H10" s="5" t="s">
         <v>15</v>
       </c>
@@ -5185,7 +5185,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="20" t="s">
         <v>68</v>
       </c>
@@ -5207,7 +5207,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="13" t="s">
         <v>0</v>
       </c>
@@ -5233,7 +5233,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>10</v>
       </c>
@@ -5260,7 +5260,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>12</v>
       </c>
@@ -5287,7 +5287,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>15</v>
       </c>
@@ -5313,7 +5313,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>21</v>
       </c>
@@ -5321,7 +5321,7 @@
         <v>13</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>33</v>
@@ -5329,7 +5329,7 @@
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B17" s="12" t="s">
         <v>22</v>
       </c>
@@ -5337,7 +5337,7 @@
         <v>79</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>33</v>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="L17" s="20"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="8" t="s">
         <v>60</v>
       </c>
@@ -5359,7 +5359,7 @@
         <v>13</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>33</v>
@@ -5377,7 +5377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H19" s="5" t="s">
         <v>10</v>
       </c>
@@ -5391,7 +5391,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="20" t="s">
         <v>69</v>
       </c>
@@ -5413,7 +5413,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="13" t="s">
         <v>0</v>
       </c>
@@ -5439,7 +5439,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="8" t="s">
         <v>28</v>
       </c>
@@ -5465,7 +5465,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="8" t="s">
         <v>30</v>
       </c>
@@ -5491,7 +5491,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="8" t="s">
         <v>26</v>
       </c>
@@ -5517,7 +5517,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="5" t="s">
         <v>20</v>
       </c>
@@ -5543,7 +5543,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
         <v>34</v>
       </c>
@@ -5569,7 +5569,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
         <v>19</v>
       </c>
@@ -5589,7 +5589,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="19" t="s">
         <v>83</v>
       </c>
@@ -5609,7 +5609,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="8" t="s">
         <v>31</v>
       </c>
@@ -5617,12 +5617,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="H30" s="20" t="s">
         <v>74</v>
@@ -5633,13 +5633,7 @@
       </c>
       <c r="L30" s="20"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B31" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>33</v>
-      </c>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H31" s="13" t="s">
         <v>23</v>
       </c>
@@ -5653,7 +5647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32"/>
       <c r="C32"/>
       <c r="D32"/>
@@ -5670,7 +5664,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33"/>
       <c r="C33"/>
       <c r="D33"/>
@@ -5687,7 +5681,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34"/>
       <c r="C34"/>
       <c r="D34"/>
@@ -5704,7 +5698,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35"/>
       <c r="C35"/>
       <c r="D35"/>
@@ -5721,7 +5715,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36"/>
       <c r="C36"/>
       <c r="D36"/>
@@ -5738,37 +5732,37 @@
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37"/>
       <c r="C37"/>
       <c r="D37"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D38"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D39"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D40"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D41"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="32" priority="30"/>
@@ -5803,10 +5797,10 @@
   <conditionalFormatting sqref="E9">
     <cfRule type="duplicateValues" dxfId="22" priority="27"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E16">
+    <cfRule type="duplicateValues" dxfId="21" priority="17"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="21" priority="17"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E18">
     <cfRule type="duplicateValues" dxfId="20" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
@@ -5877,13 +5871,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5EE4785-03B3-42C8-BF36-D812A392D9B8}">
   <sheetPr codeName="Hoja4"/>
   <dimension ref="A1:B25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="95.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="95.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="47.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="94.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="94.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>35</v>
       </c>
@@ -5891,7 +5885,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>6</v>
       </c>
@@ -5899,7 +5893,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -5907,7 +5901,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>9</v>
       </c>
@@ -5915,7 +5909,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>20</v>
       </c>
@@ -5923,7 +5917,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>19</v>
       </c>
@@ -5931,7 +5925,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>7</v>
       </c>
@@ -5939,7 +5933,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>43</v>
       </c>
@@ -5947,7 +5941,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>8</v>
       </c>
@@ -5955,7 +5949,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>14</v>
       </c>
@@ -5963,7 +5957,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>12</v>
       </c>
@@ -5971,7 +5965,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>61</v>
       </c>
@@ -5979,7 +5973,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>21</v>
       </c>
@@ -5987,7 +5981,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>48</v>
       </c>
@@ -5995,7 +5989,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>10</v>
       </c>
@@ -6003,7 +5997,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>26</v>
       </c>
@@ -6011,7 +6005,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
         <v>32</v>
       </c>
@@ -6019,7 +6013,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
         <v>30</v>
       </c>
@@ -6027,7 +6021,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
         <v>34</v>
       </c>
@@ -6035,7 +6029,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="150" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="144" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
         <v>28</v>
       </c>
@@ -6043,7 +6037,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>31</v>
       </c>
@@ -6051,7 +6045,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>27</v>
       </c>
@@ -6059,7 +6053,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
         <v>18</v>
       </c>
@@ -6067,7 +6061,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A24" s="10" t="s">
         <v>11</v>
       </c>
@@ -6075,7 +6069,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="10" t="s">
         <v>64</v>
       </c>
@@ -6090,21 +6084,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -6305,32 +6284,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6347,4 +6316,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - sáb 01/08/2026 10:07:19,12
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Julio.xlsx
+++ b/Cronograma de Tareas/Cronograma Julio.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AD3C06B-D3A5-469F-9D12-146835E6C5F7}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5E7A2BB-6929-475C-98DB-39214E963A4A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="85">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -320,6 +320,9 @@
   </si>
   <si>
     <t>Revisión Usuarios Nivel 2 - CRM con TAG de Abuso de Bonos (15 días)</t>
+  </si>
+  <si>
+    <t>Sebastian Hincapié</t>
   </si>
 </sst>
 </file>
@@ -2986,18 +2989,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="130" priority="30"/>
@@ -4833,18 +4836,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="65" priority="30"/>
@@ -5058,13 +5061,13 @@
         <v>10</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.3">
@@ -5110,13 +5113,13 @@
         <v>60</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="K7" s="8" t="s">
         <v>60</v>
       </c>
       <c r="L7" s="14" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.3">
@@ -5162,13 +5165,13 @@
         <v>6</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>6</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.3">
@@ -5198,13 +5201,13 @@
         <v>7</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>7</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.3">
@@ -5251,13 +5254,13 @@
         <v>14</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="K13" s="5" t="s">
         <v>14</v>
       </c>
       <c r="L13" s="14" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.3">
@@ -5304,13 +5307,13 @@
         <v>20</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>20</v>
       </c>
       <c r="L15" s="14" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.3">
@@ -5751,18 +5754,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="32" priority="30"/>
@@ -6285,18 +6288,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6319,14 +6322,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -6341,4 +6336,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>